<commit_message>
added wave transmission as a supported response.
</commit_message>
<xml_diff>
--- a/SS_floodwall_input.xlsx
+++ b/SS_floodwall_input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0_StormSim_Task\Task_FY25_NCMP_Part_1\Exceedance_code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0_StormSim_Task\StormSim-Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5182B439-F5A2-454A-88E9-CF4FD6AB4B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E4226C9-3649-47D9-83E9-0BA3CA327E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{392BD468-0951-485E-9EDB-F7D879C79477}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{392BD468-0951-485E-9EDB-F7D879C79477}"/>
   </bookViews>
   <sheets>
     <sheet name="FloodWall" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="168">
   <si>
     <t>NA</t>
   </si>
@@ -531,6 +531,15 @@
   </si>
   <si>
     <t>StormSim Project General Inputs</t>
+  </si>
+  <si>
+    <t>calc_wave_transmission</t>
+  </si>
+  <si>
+    <t>compute_wave_transmission</t>
+  </si>
+  <si>
+    <t>Compute wave transmission (eurotop)</t>
   </si>
 </sst>
 </file>
@@ -540,7 +549,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -582,6 +591,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="13">
@@ -844,7 +859,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -985,6 +1000,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="3"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1301,7 +1319,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FDE711C-012D-4C9C-BCEB-7FA13A47BF68}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="101.7109375" customWidth="1"/>
@@ -2332,10 +2350,10 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
-        <v>14</v>
+        <v>166</v>
       </c>
       <c r="B53" s="12" t="s">
-        <v>13</v>
+        <v>167</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>0</v>
@@ -2346,66 +2364,66 @@
     </row>
     <row r="54" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C54" s="11" t="s">
         <v>0</v>
       </c>
       <c r="D54" s="10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B55" s="12" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C55" s="11" t="s">
         <v>0</v>
       </c>
       <c r="D55" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C56" s="11" t="s">
         <v>0</v>
       </c>
       <c r="D56" s="10">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B57" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="D57" s="6">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="B57" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D57" s="10">
+        <v>8</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C58" s="7" t="s">
         <v>0</v>
@@ -2414,27 +2432,45 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="5" t="s">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D59" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B60" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C59" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D59" s="2">
+      <c r="C60" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D60" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="1"/>
-      <c r="B60" s="1"/>
-      <c r="C60" s="1"/>
-      <c r="D60" s="1"/>
-    </row>
-    <row r="61" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1"/>
+      <c r="B61" s="1"/>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="60" t="s">
+        <v>165</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>

</xml_diff>